<commit_message>
Add IRR index analysis and update figures
Introduced ScriptAnalysis/7_a_IRR_index.R for IRR index analysis and group recovery time visualization. Updated and added several figures (fig4, fig5_a) and their data, removed obsolete figures (fig7-fig12), and refactored panel plotting functions by moving them from 6_b_visualization.R to function/forecast.R. Minor update in 6_a_forecast.R to include Shortname in output.
</commit_message>
<xml_diff>
--- a/Outcome/Publish/figure_data/fig4.xlsx
+++ b/Outcome/Publish/figure_data/fig4.xlsx
@@ -204,9 +204,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -243,7 +241,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>

<commit_message>
Add and update figures and recovery analysis for fig5
Introduces new files for fig5 (afdesign, pdf, png, and data), updates fig4 and related data, and refactors R scripts to support group-level recovery metrics and visualization. The changes include enhanced calculation and display of recovery/balance periods, improved plotting functions, and updated output dimensions for figures. Also updates figure data exports and underlying model outputs to reflect these improvements.
</commit_message>
<xml_diff>
--- a/Outcome/Publish/figure_data/fig4.xlsx
+++ b/Outcome/Publish/figure_data/fig4.xlsx
@@ -207,9 +207,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -246,7 +244,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>

<commit_message>
Enhance seasonality analysis and visualization in IRR script
Refactored ScriptAnalysis/6_a_IRR_index.R to improve seasonality analysis by adding amplitude metrics, robust phase shift calculations (including centre-of-mass peak detection), and updated radar chart visualization with clearer peak markers. Updated figure files and data to reflect these changes and clarified period definitions for post-pandemic analysis.
</commit_message>
<xml_diff>
--- a/Outcome/Publish/figure_data/fig4.xlsx
+++ b/Outcome/Publish/figure_data/fig4.xlsx
@@ -161,19 +161,17 @@
     <t xml:space="preserve">Pre-COVID (Observed)</t>
   </si>
   <si>
-    <t xml:space="preserve">Post-Recovery (Observed)</t>
+    <t xml:space="preserve">Post-PHSM (Observed)</t>
   </si>
   <si>
-    <t xml:space="preserve">Post-Recovery (Predicted)</t>
+    <t xml:space="preserve">Post-PHSM (Predicted)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -210,7 +208,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>